<commit_message>
feat(thesis): pre-version for the supervisor after the user's two readings; the revision of all 113 remarks, the pocket series as the main case of 5.2 to 5.5 and 7, the after-test contour scans (M5, contour_wear.py: axis from the GINA circles, fillet rotation, wear 46 to 197 µm, onset 25,42 to 25,45 mm), the damage pictures in 6.2, the reviewer round (63 findings), semicolons and colons out of the prose, the regenerated figures with the grid behind, the measured-geometry decks (ADR-116 item 54, ADR-118 amendments of 2026-10-21, roadmap M5 and T4)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/70_input/72_Kleingetriebepruefstand_KV3/kst-E_Laufversuche_KV3.xlsx
+++ b/70_input/72_Kleingetriebepruefstand_KV3/kst-E_Laufversuche_KV3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub-tkuhn39\semesterthesis\70_input\72_Kleingetriebepruefstand_KV3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98D51430-287A-45D1-8DC7-9A3CD7F5BD23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AA3F3D2-2F77-4BAF-938D-4B350E82F015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{09DE1DE6-8CB8-D84C-8367-607651AAD6B1}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{09DE1DE6-8CB8-D84C-8367-607651AAD6B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="280">
   <si>
     <t>A</t>
   </si>
@@ -982,6 +982,15 @@
   </si>
   <si>
     <t>sehr schwankend("ssc"): Stopp nach 2min (2 327), (ab ssc: 13,3…15,7bzw16,0Nm) (auch später: 13,1…15,0Nm) bis 36 349; (ab 13,9Nm…15,7Nm:) 304 112; (ab 13,4…15,8Nm:) 1 019 086; (ab 13,5…15,8Nm:) 1 909 028; (ab 14,0…15,4Nm:) 1 963 654; (ab 14,0...15,1:) 2 034 128</t>
+  </si>
+  <si>
+    <t>kst-E_76</t>
+  </si>
+  <si>
+    <t>... 6,8 Nm -&gt; nachverspannt auf ... Nm bei TA ... °C, TP ... °C ;  (ca. ... Nm Verlust über ...) Bilder ... . Noch/Schon ... Anrisse. Verschleiß ... erkennbar.
+... 6,8 Nm -&gt; nachverspannt auf ... Nm bei TA ... °C, TP ... °C ;  (ca. ... Nm Verlust über ...) Bilder ... . Noch/Schon ... Anrisse. Verschleiß ... erkennbar.
+... 6,8 Nm -&gt; nachverspannt auf ... Nm bei TA ... °C, TP ... °C ;  (ca. ... Nm Verlust über ...) Bilder ... . Noch/Schon ... Anrisse. Verschleiß ... erkennbar.
+... 6,8 Nm -&gt; nachverspannt auf ... Nm bei TA ... °C, TP ... °C ;  (ca. ... Nm Verlust über ...) Bilder ... . Noch/Schon ... Anrisse. Verschleiß ... erkennbar.</t>
   </si>
 </sst>
 </file>
@@ -2014,32 +2023,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C3A9485-4D50-0041-9D5B-E8D35C0F1538}">
   <dimension ref="A1:U103"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="4.6640625" customWidth="1"/>
+    <col min="3" max="3" width="4.625" customWidth="1"/>
     <col min="4" max="4" width="10.5" customWidth="1"/>
-    <col min="5" max="5" width="6.83203125" customWidth="1"/>
+    <col min="5" max="5" width="6.875" customWidth="1"/>
     <col min="6" max="6" width="9.5" customWidth="1"/>
-    <col min="7" max="7" width="5.33203125" customWidth="1"/>
-    <col min="8" max="8" width="10.1640625" style="157" customWidth="1"/>
+    <col min="7" max="7" width="5.375" customWidth="1"/>
+    <col min="8" max="8" width="10.125" style="157" customWidth="1"/>
     <col min="9" max="9" width="5.5" customWidth="1"/>
-    <col min="10" max="10" width="26.83203125" customWidth="1"/>
-    <col min="11" max="11" width="8.6640625" customWidth="1"/>
-    <col min="12" max="12" width="8.1640625" customWidth="1"/>
-    <col min="13" max="13" width="19.83203125" customWidth="1"/>
-    <col min="14" max="14" width="19.1640625" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
-    <col min="16" max="16" width="4.1640625" customWidth="1"/>
-    <col min="17" max="17" width="10.33203125" customWidth="1"/>
-    <col min="18" max="18" width="9.1640625" customWidth="1"/>
+    <col min="10" max="10" width="26.875" customWidth="1"/>
+    <col min="11" max="11" width="8.625" customWidth="1"/>
+    <col min="12" max="12" width="8.125" customWidth="1"/>
+    <col min="13" max="13" width="19.875" customWidth="1"/>
+    <col min="14" max="14" width="19.125" customWidth="1"/>
+    <col min="15" max="15" width="12.875" customWidth="1"/>
+    <col min="16" max="16" width="4.125" customWidth="1"/>
+    <col min="17" max="17" width="10.375" customWidth="1"/>
+    <col min="18" max="18" width="9.125" customWidth="1"/>
     <col min="19" max="19" width="13.5" customWidth="1"/>
     <col min="20" max="20" width="148" style="158" customWidth="1"/>
     <col min="21" max="21" width="195.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="61.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:21" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2102,7 +2111,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:21" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" s="5" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>20</v>
       </c>
@@ -2145,7 +2154,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:21" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" s="5" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>25</v>
       </c>
@@ -2185,7 +2194,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:21" s="5" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" s="5" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>26</v>
       </c>
@@ -2225,7 +2234,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:21" s="9" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" s="9" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>28</v>
       </c>
@@ -2265,7 +2274,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:21" s="9" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" s="9" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>31</v>
       </c>
@@ -2306,7 +2315,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:21" s="5" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" s="5" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>33</v>
       </c>
@@ -2362,7 +2371,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:21" s="14" customFormat="1" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:21" s="14" customFormat="1" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
         <v>36</v>
       </c>
@@ -2418,7 +2427,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:21" s="22" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:21" s="22" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="20" t="s">
         <v>38</v>
       </c>
@@ -2475,7 +2484,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:21" s="29" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:21" s="29" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
         <v>42</v>
       </c>
@@ -2535,7 +2544,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:21" s="36" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:21" s="36" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="34" t="s">
         <v>45</v>
       </c>
@@ -2595,7 +2604,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:21" s="29" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:21" s="29" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>48</v>
       </c>
@@ -2655,7 +2664,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:21" s="36" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:21" s="36" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="34" t="s">
         <v>51</v>
       </c>
@@ -2715,7 +2724,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="14" spans="1:21" s="36" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:21" s="36" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="34" t="s">
         <v>54</v>
       </c>
@@ -2775,7 +2784,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:21" s="36" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:21" s="36" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="34" t="s">
         <v>57</v>
       </c>
@@ -2835,7 +2844,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="16" spans="1:21" s="36" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:21" s="36" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="34" t="s">
         <v>61</v>
       </c>
@@ -2895,7 +2904,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="17" spans="1:20" s="36" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:20" s="36" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="34" t="s">
         <v>65</v>
       </c>
@@ -2955,7 +2964,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:20" s="36" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:20" s="36" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="34" t="s">
         <v>68</v>
       </c>
@@ -3015,7 +3024,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="19" spans="1:20" s="36" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:20" s="36" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="34" t="s">
         <v>71</v>
       </c>
@@ -3075,7 +3084,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="20" spans="1:20" s="48" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:20" s="48" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="46" t="s">
         <v>74</v>
       </c>
@@ -3135,7 +3144,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:20" s="53" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:20" s="53" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="51" t="s">
         <v>78</v>
       </c>
@@ -3195,7 +3204,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:20" s="36" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:20" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="34" t="s">
         <v>81</v>
       </c>
@@ -3255,7 +3264,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="23" spans="1:20" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:20" s="5" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="57" t="s">
         <v>84</v>
       </c>
@@ -3315,7 +3324,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="24" spans="1:20" s="40" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:20" s="40" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="64" t="s">
         <v>88</v>
       </c>
@@ -3375,7 +3384,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="25" spans="1:20" s="74" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:20" s="74" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="70" t="s">
         <v>92</v>
       </c>
@@ -3435,7 +3444,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="26" spans="1:20" s="82" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:20" s="82" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="78" t="s">
         <v>96</v>
       </c>
@@ -3495,7 +3504,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="27" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="85" t="s">
         <v>100</v>
       </c>
@@ -3555,7 +3564,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="28" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="85" t="s">
         <v>103</v>
       </c>
@@ -3615,7 +3624,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="29" spans="1:20" s="93" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:20" s="93" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="91" t="s">
         <v>106</v>
       </c>
@@ -3675,7 +3684,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="30" spans="1:20" s="93" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:20" s="93" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="91" t="s">
         <v>110</v>
       </c>
@@ -3735,7 +3744,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="31" spans="1:20" s="74" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:20" s="74" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="70" t="s">
         <v>115</v>
       </c>
@@ -3795,7 +3804,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="32" spans="1:20" s="101" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:20" s="101" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="99" t="s">
         <v>119</v>
       </c>
@@ -3855,7 +3864,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="33" spans="1:20" s="108" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:20" s="108" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="106" t="s">
         <v>122</v>
       </c>
@@ -3915,7 +3924,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="34" spans="1:20" s="114" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:20" s="114" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="112" t="s">
         <v>125</v>
       </c>
@@ -3975,7 +3984,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="35" spans="1:20" s="121" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:20" s="121" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="118" t="s">
         <v>130</v>
       </c>
@@ -4035,7 +4044,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="36" spans="1:20" s="114" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:20" s="114" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="112" t="s">
         <v>133</v>
       </c>
@@ -4095,7 +4104,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="37" spans="1:20" s="30" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:20" s="30" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="85" t="s">
         <v>140</v>
       </c>
@@ -4155,7 +4164,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="38" spans="1:20" s="30" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:20" s="30" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="85" t="s">
         <v>143</v>
       </c>
@@ -4215,7 +4224,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="39" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:20" s="30" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="85" t="s">
         <v>147</v>
       </c>
@@ -4275,7 +4284,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="40" spans="1:20" s="40" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:20" s="40" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="64" t="s">
         <v>150</v>
       </c>
@@ -4335,7 +4344,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="41" spans="1:20" s="40" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:20" s="40" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="64" t="s">
         <v>154</v>
       </c>
@@ -4395,7 +4404,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="42" spans="1:20" s="40" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:20" s="40" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="40" t="s">
         <v>157</v>
       </c>
@@ -4456,7 +4465,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="43" spans="1:20" s="82" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:20" s="82" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="78" t="s">
         <v>160</v>
       </c>
@@ -4516,7 +4525,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="44" spans="1:20" s="134" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:20" s="134" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="40" t="s">
         <v>163</v>
       </c>
@@ -4569,7 +4578,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="45" spans="1:20" s="36" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:20" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="36" t="s">
         <v>165</v>
       </c>
@@ -4605,7 +4614,7 @@
       </c>
       <c r="T45" s="38"/>
     </row>
-    <row r="46" spans="1:20" s="114" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:20" s="114" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="114" t="s">
         <v>166</v>
       </c>
@@ -4642,7 +4651,7 @@
       </c>
       <c r="T46" s="116"/>
     </row>
-    <row r="47" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="135" t="s">
         <v>167</v>
       </c>
@@ -4666,7 +4675,7 @@
       </c>
       <c r="T47" s="139"/>
     </row>
-    <row r="48" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="135" t="s">
         <v>168</v>
       </c>
@@ -4690,7 +4699,7 @@
       </c>
       <c r="T48" s="139"/>
     </row>
-    <row r="49" spans="1:20" s="135" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:20" s="135" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="135" t="s">
         <v>169</v>
       </c>
@@ -4715,7 +4724,7 @@
       </c>
       <c r="T49" s="139"/>
     </row>
-    <row r="50" spans="1:20" s="135" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:20" s="135" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="135" t="s">
         <v>170</v>
       </c>
@@ -4741,7 +4750,7 @@
       <c r="R50" s="142"/>
       <c r="T50" s="139"/>
     </row>
-    <row r="51" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="135" t="s">
         <v>171</v>
       </c>
@@ -4795,7 +4804,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="52" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="135" t="s">
         <v>176</v>
       </c>
@@ -4849,7 +4858,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="53" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="135" t="s">
         <v>178</v>
       </c>
@@ -4903,7 +4912,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="54" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="135" t="s">
         <v>180</v>
       </c>
@@ -4958,7 +4967,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="55" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="135" t="s">
         <v>184</v>
       </c>
@@ -4986,7 +4995,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="56" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="135" t="s">
         <v>185</v>
       </c>
@@ -5010,7 +5019,7 @@
       </c>
       <c r="T56" s="139"/>
     </row>
-    <row r="57" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="135" t="s">
         <v>186</v>
       </c>
@@ -5034,7 +5043,7 @@
       </c>
       <c r="T57" s="139"/>
     </row>
-    <row r="58" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="135" t="s">
         <v>187</v>
       </c>
@@ -5058,7 +5067,7 @@
       </c>
       <c r="T58" s="139"/>
     </row>
-    <row r="59" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="135" t="s">
         <v>188</v>
       </c>
@@ -5083,7 +5092,7 @@
       </c>
       <c r="T59" s="139"/>
     </row>
-    <row r="60" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="135" t="s">
         <v>189</v>
       </c>
@@ -5109,7 +5118,7 @@
       <c r="R60" s="142"/>
       <c r="T60" s="139"/>
     </row>
-    <row r="61" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="135" t="s">
         <v>190</v>
       </c>
@@ -5133,7 +5142,7 @@
       </c>
       <c r="T61" s="139"/>
     </row>
-    <row r="62" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="135" t="s">
         <v>191</v>
       </c>
@@ -5157,7 +5166,7 @@
       </c>
       <c r="T62" s="139"/>
     </row>
-    <row r="63" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="135" t="s">
         <v>192</v>
       </c>
@@ -5181,7 +5190,7 @@
       </c>
       <c r="T63" s="139"/>
     </row>
-    <row r="64" spans="1:20" s="143" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:20" s="143" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="135" t="s">
         <v>184</v>
       </c>
@@ -5236,7 +5245,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="65" spans="1:20" s="143" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:20" s="143" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="135" t="s">
         <v>185</v>
       </c>
@@ -5293,7 +5302,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="66" spans="1:20" s="143" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:20" s="143" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="135" t="s">
         <v>186</v>
       </c>
@@ -5348,7 +5357,7 @@
       </c>
       <c r="T66" s="139"/>
     </row>
-    <row r="67" spans="1:20" s="143" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:20" s="143" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="135" t="s">
         <v>187</v>
       </c>
@@ -5407,7 +5416,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="68" spans="1:20" s="143" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:20" s="143" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="135" t="s">
         <v>188</v>
       </c>
@@ -5464,7 +5473,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="69" spans="1:20" s="143" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:20" s="143" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="135" t="s">
         <v>189</v>
       </c>
@@ -5523,7 +5532,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A70" s="135" t="s">
         <v>190</v>
       </c>
@@ -5582,7 +5591,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A71" s="144" t="s">
         <v>191</v>
       </c>
@@ -5641,7 +5650,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="72" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="135" t="s">
         <v>188</v>
       </c>
@@ -5674,7 +5683,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="73" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="135" t="s">
         <v>189</v>
       </c>
@@ -5705,7 +5714,7 @@
       </c>
       <c r="T73" s="160"/>
     </row>
-    <row r="74" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="135" t="s">
         <v>190</v>
       </c>
@@ -5736,7 +5745,7 @@
       </c>
       <c r="T74" s="161"/>
     </row>
-    <row r="75" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="135" t="s">
         <v>191</v>
       </c>
@@ -5770,7 +5779,7 @@
       </c>
       <c r="T75" s="139"/>
     </row>
-    <row r="76" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:20" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="135" t="s">
         <v>192</v>
       </c>
@@ -5821,7 +5830,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="77" spans="1:20" s="148" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:20" s="148" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="148" t="s">
         <v>210</v>
       </c>
@@ -5869,7 +5878,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="78" spans="1:20" s="148" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:20" s="148" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B78" s="149">
         <v>46252</v>
       </c>
@@ -5914,7 +5923,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="79" spans="1:20" s="148" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:20" s="148" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B79" s="149">
         <v>46252</v>
       </c>
@@ -5956,7 +5965,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="80" spans="1:20" s="148" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:20" s="148" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B80" s="149">
         <v>46252</v>
       </c>
@@ -5998,7 +6007,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="81" spans="1:21" s="148" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:21" s="148" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B81" s="149">
         <v>46253</v>
       </c>
@@ -6043,7 +6052,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="82" spans="1:21" s="148" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:21" s="148" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B82" s="149">
         <v>46253</v>
       </c>
@@ -6088,7 +6097,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="83" spans="1:21" s="148" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:21" s="148" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B83" s="149">
         <v>46255</v>
       </c>
@@ -6120,7 +6129,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="84" spans="1:21" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:21" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="135" t="s">
         <v>230</v>
       </c>
@@ -6168,7 +6177,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="85" spans="1:21" s="135" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:21" s="135" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="135" t="s">
         <v>232</v>
       </c>
@@ -6219,7 +6228,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="86" spans="1:21" s="148" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:21" s="148" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A86" s="148" t="s">
         <v>234</v>
       </c>
@@ -6267,7 +6276,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="87" spans="1:21" s="143" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:21" s="143" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="153" t="s">
         <v>238</v>
       </c>
@@ -6319,7 +6328,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="88" spans="1:21" s="148" customFormat="1" ht="48" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:21" s="148" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A88" s="148" t="s">
         <v>240</v>
       </c>
@@ -6373,7 +6382,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="89" spans="1:21" s="148" customFormat="1" ht="240" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:21" s="148" customFormat="1" ht="236.25" x14ac:dyDescent="0.25">
       <c r="A89" s="148" t="s">
         <v>245</v>
       </c>
@@ -6430,7 +6439,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="90" spans="1:21" s="148" customFormat="1" ht="48" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:21" s="148" customFormat="1" ht="63" x14ac:dyDescent="0.25">
       <c r="A90" s="148" t="s">
         <v>251</v>
       </c>
@@ -6487,7 +6496,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="91" spans="1:21" s="148" customFormat="1" ht="240" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:21" s="148" customFormat="1" ht="236.25" x14ac:dyDescent="0.25">
       <c r="A91" s="148" t="s">
         <v>254</v>
       </c>
@@ -6544,7 +6553,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="92" spans="1:21" s="148" customFormat="1" ht="160" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:21" s="148" customFormat="1" ht="157.5" x14ac:dyDescent="0.25">
       <c r="A92" s="148" t="s">
         <v>257</v>
       </c>
@@ -6601,7 +6610,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="93" spans="1:21" s="148" customFormat="1" ht="128" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:21" s="148" customFormat="1" ht="141.75" x14ac:dyDescent="0.25">
       <c r="A93" s="148" t="s">
         <v>262</v>
       </c>
@@ -6655,7 +6664,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="94" spans="1:21" s="148" customFormat="1" ht="256" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:21" s="148" customFormat="1" ht="252" x14ac:dyDescent="0.25">
       <c r="A94" s="148" t="s">
         <v>267</v>
       </c>
@@ -6712,7 +6721,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="95" spans="1:21" s="148" customFormat="1" ht="272" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:21" s="148" customFormat="1" ht="283.5" x14ac:dyDescent="0.25">
       <c r="A95" s="148" t="s">
         <v>271</v>
       </c>
@@ -6765,12 +6774,52 @@
       </c>
       <c r="U95" s="156"/>
     </row>
-    <row r="97" spans="20:20" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:21" s="148" customFormat="1" ht="63" x14ac:dyDescent="0.25">
+      <c r="A96" s="148" t="s">
+        <v>278</v>
+      </c>
+      <c r="B96" s="149"/>
+      <c r="C96" s="148" t="s">
+        <v>172</v>
+      </c>
+      <c r="D96" s="148" t="s">
+        <v>211</v>
+      </c>
+      <c r="E96" s="148">
+        <v>95919</v>
+      </c>
+      <c r="F96" s="148">
+        <v>97361</v>
+      </c>
+      <c r="G96" s="148">
+        <v>75</v>
+      </c>
+      <c r="H96" s="150">
+        <v>80</v>
+      </c>
+      <c r="J96" s="156"/>
+      <c r="K96" s="148">
+        <v>7.8</v>
+      </c>
+      <c r="M96" s="156"/>
+      <c r="Q96" s="148">
+        <f>K96*(52/51)</f>
+        <v>7.9529411764705875</v>
+      </c>
+      <c r="R96" s="148">
+        <v>3058</v>
+      </c>
+      <c r="T96" s="152" t="s">
+        <v>279</v>
+      </c>
+      <c r="U96" s="156"/>
+    </row>
+    <row r="97" spans="20:20" x14ac:dyDescent="0.25">
       <c r="T97" s="158" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="103" spans="20:20" x14ac:dyDescent="0.4">
+    <row r="103" spans="20:20" x14ac:dyDescent="0.25">
       <c r="T103" s="158" t="s">
         <v>216</v>
       </c>

</xml_diff>